<commit_message>
adding this weeks sw results
</commit_message>
<xml_diff>
--- a/data/The_Last_Man-tis_on_Earth.xlsx
+++ b/data/The_Last_Man-tis_on_Earth.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tom\Documents\website\rhytididae\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F13F0BC-09E1-48E2-8E44-B5788D8A55FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B8CB4B8-3C51-47D5-908E-243AD77B91EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="40180" yWindow="1780" windowWidth="28800" windowHeight="15370" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="204">
   <si>
     <t>Survey Name</t>
   </si>
@@ -982,9 +982,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -992,7 +992,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -1000,7 +1000,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -1008,7 +1008,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -1016,7 +1016,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -1024,7 +1024,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -1040,29 +1040,29 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C94"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -1073,7 +1073,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>17</v>
       </c>
@@ -1084,7 +1084,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>20</v>
       </c>
@@ -1095,7 +1095,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>23</v>
       </c>
@@ -1106,7 +1106,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>26</v>
       </c>
@@ -1114,17 +1114,17 @@
         <v>27</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>14</v>
       </c>
@@ -1135,7 +1135,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>30</v>
       </c>
@@ -1146,7 +1146,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>31</v>
       </c>
@@ -1157,7 +1157,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>32</v>
       </c>
@@ -1168,7 +1168,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>33</v>
       </c>
@@ -1179,7 +1179,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>34</v>
       </c>
@@ -1190,7 +1190,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>35</v>
       </c>
@@ -1201,7 +1201,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>36</v>
       </c>
@@ -1212,7 +1212,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>37</v>
       </c>
@@ -1223,7 +1223,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>38</v>
       </c>
@@ -1234,7 +1234,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>39</v>
       </c>
@@ -1245,7 +1245,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>40</v>
       </c>
@@ -1256,7 +1256,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>41</v>
       </c>
@@ -1267,7 +1267,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>42</v>
       </c>
@@ -1278,7 +1278,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>43</v>
       </c>
@@ -1289,7 +1289,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>44</v>
       </c>
@@ -1300,7 +1300,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>45</v>
       </c>
@@ -1311,7 +1311,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>46</v>
       </c>
@@ -1322,7 +1322,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>47</v>
       </c>
@@ -1333,7 +1333,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>48</v>
       </c>
@@ -1344,7 +1344,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>49</v>
       </c>
@@ -1355,7 +1355,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>50</v>
       </c>
@@ -1366,7 +1366,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>51</v>
       </c>
@@ -1377,7 +1377,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>52</v>
       </c>
@@ -1388,7 +1388,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>53</v>
       </c>
@@ -1399,7 +1399,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>54</v>
       </c>
@@ -1410,7 +1410,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>26</v>
       </c>
@@ -1418,17 +1418,17 @@
         <v>27</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>14</v>
       </c>
@@ -1439,7 +1439,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>57</v>
       </c>
@@ -1450,7 +1450,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>58</v>
       </c>
@@ -1461,7 +1461,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>59</v>
       </c>
@@ -1472,7 +1472,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>60</v>
       </c>
@@ -1483,7 +1483,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>61</v>
       </c>
@@ -1494,7 +1494,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>62</v>
       </c>
@@ -1505,7 +1505,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>63</v>
       </c>
@@ -1516,7 +1516,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>64</v>
       </c>
@@ -1527,7 +1527,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>65</v>
       </c>
@@ -1538,7 +1538,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>66</v>
       </c>
@@ -1549,7 +1549,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>67</v>
       </c>
@@ -1560,7 +1560,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>68</v>
       </c>
@@ -1571,7 +1571,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>69</v>
       </c>
@@ -1582,7 +1582,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>70</v>
       </c>
@@ -1593,7 +1593,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>71</v>
       </c>
@@ -1604,7 +1604,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>35</v>
       </c>
@@ -1615,7 +1615,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>72</v>
       </c>
@@ -1626,7 +1626,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>73</v>
       </c>
@@ -1637,7 +1637,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>74</v>
       </c>
@@ -1648,7 +1648,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>75</v>
       </c>
@@ -1659,7 +1659,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>76</v>
       </c>
@@ -1670,7 +1670,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>77</v>
       </c>
@@ -1681,7 +1681,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>78</v>
       </c>
@@ -1692,7 +1692,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>79</v>
       </c>
@@ -1703,7 +1703,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>26</v>
       </c>
@@ -1711,22 +1711,22 @@
         <v>27</v>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>14</v>
       </c>
@@ -1737,17 +1737,17 @@
         <v>16</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>14</v>
       </c>
@@ -1758,7 +1758,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>83</v>
       </c>
@@ -1771,9 +1771,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:K26"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="8" max="8" width="9.81640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>85</v>
       </c>
@@ -1805,7 +1808,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
         <v>46178.563839226612</v>
       </c>
@@ -1840,7 +1843,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
         <v>46178.611560342382</v>
       </c>
@@ -1872,7 +1875,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
         <v>46178.645161778601</v>
       </c>
@@ -1904,7 +1907,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
         <v>46178.648832837462</v>
       </c>
@@ -1936,7 +1939,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
         <v>46178.706171497193</v>
       </c>
@@ -1968,7 +1971,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
         <v>46178.719022849597</v>
       </c>
@@ -1990,8 +1993,8 @@
       <c r="G7" t="s">
         <v>17</v>
       </c>
-      <c r="H7" t="s">
-        <v>32</v>
+      <c r="H7">
+        <v>268077845</v>
       </c>
       <c r="I7" t="s">
         <v>79</v>
@@ -2000,7 +2003,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" s="1">
         <v>46178.785269131098</v>
       </c>
@@ -2032,7 +2035,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" s="1">
         <v>46179.021981183287</v>
       </c>
@@ -2064,7 +2067,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" s="1">
         <v>46179.050878479109</v>
       </c>
@@ -2096,7 +2099,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" s="1">
         <v>46179.169924163252</v>
       </c>
@@ -2128,7 +2131,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" s="1">
         <v>46179.421458056233</v>
       </c>
@@ -2160,7 +2163,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" s="1">
         <v>46179.541931204789</v>
       </c>
@@ -2192,7 +2195,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" s="1">
         <v>46179.865207506722</v>
       </c>
@@ -2224,7 +2227,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" s="1">
         <v>46179.920047726409</v>
       </c>
@@ -2256,7 +2259,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A16" s="1">
         <v>46179.958327778193</v>
       </c>
@@ -2288,7 +2291,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" s="1">
         <v>46180.149676061257</v>
       </c>
@@ -2320,7 +2323,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" s="1">
         <v>46180.277126003217</v>
       </c>
@@ -2352,7 +2355,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" s="1">
         <v>46180.602121176889</v>
       </c>
@@ -2384,7 +2387,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" s="1">
         <v>46182.883224256759</v>
       </c>
@@ -2416,7 +2419,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" s="1">
         <v>46182.893500736704</v>
       </c>
@@ -2448,7 +2451,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22" s="1">
         <v>46182.910639658621</v>
       </c>
@@ -2480,7 +2483,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" s="1">
         <v>46182.972886263407</v>
       </c>
@@ -2512,7 +2515,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24" s="1">
         <v>46183.000450496598</v>
       </c>
@@ -2544,7 +2547,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25" s="1">
         <v>46183.005973159561</v>
       </c>
@@ -2576,7 +2579,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" s="1">
         <v>46183.425911745697</v>
       </c>

</xml_diff>